<commit_message>
Co-authored-by: Habiba Ratna Safitri <ratnarealme666-netizen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/pesanan.xlsx
+++ b/pesanan.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,6 +523,28 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>30.000 - 1.000.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bucket Snack Ceria</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>40.000 - 300.000</t>
         </is>
       </c>
     </row>

</xml_diff>